<commit_message>
fim entire run 9.30
</commit_message>
<xml_diff>
--- a/data/monthly_state_ui.xlsx
+++ b/data/monthly_state_ui.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R680"/>
+  <dimension ref="A1:R681"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
@@ -3032,7 +3032,7 @@
         <v>368829</v>
       </c>
       <c r="F65">
-        <v>17326080</v>
+        <v>16491139</v>
       </c>
       <c r="G65">
         <v>19257888</v>
@@ -3041,7 +3041,7 @@
         <v>1299524</v>
       </c>
       <c r="I65">
-        <v>69.06999999999999</v>
+        <v>60.49</v>
       </c>
       <c r="J65">
         <v>35.92</v>
@@ -36368,7 +36368,7 @@
         <v>46142</v>
       </c>
       <c r="B677">
-        <v>849594</v>
+        <v>849491</v>
       </c>
       <c r="C677">
         <v>1750.1</v>
@@ -36380,7 +36380,7 @@
         <v>175582</v>
       </c>
       <c r="F677">
-        <v>7443594</v>
+        <v>7443591</v>
       </c>
       <c r="G677">
         <v>6573847</v>
@@ -36424,7 +36424,7 @@
         <v>46173</v>
       </c>
       <c r="B678">
-        <v>808326</v>
+        <v>808156</v>
       </c>
       <c r="C678">
         <v>1640</v>
@@ -36436,7 +36436,7 @@
         <v>176316</v>
       </c>
       <c r="F678">
-        <v>7303006</v>
+        <v>7303000</v>
       </c>
       <c r="G678">
         <v>5941902</v>
@@ -36472,7 +36472,7 @@
         <v>15181</v>
       </c>
       <c r="R678">
-        <v>501948</v>
+        <v>502197</v>
       </c>
     </row>
     <row r="679">
@@ -36480,31 +36480,31 @@
         <v>46203</v>
       </c>
       <c r="B679">
-        <v>961399</v>
+        <v>961311</v>
       </c>
       <c r="C679">
         <v>1702.4</v>
       </c>
       <c r="D679">
-        <v>438099</v>
+        <v>437550</v>
       </c>
       <c r="E679">
-        <v>169553</v>
+        <v>168067</v>
       </c>
       <c r="F679">
-        <v>7477470</v>
+        <v>7469238</v>
       </c>
       <c r="G679">
-        <v>6613638</v>
+        <v>6608669</v>
       </c>
       <c r="H679">
-        <v>3189438</v>
+        <v>3187229</v>
       </c>
       <c r="I679">
-        <v>494.08</v>
+        <v>494.09</v>
       </c>
       <c r="J679">
-        <v>39.36</v>
+        <v>39.33</v>
       </c>
       <c r="K679">
         <v>15.74</v>
@@ -36513,22 +36513,22 @@
         <v>488.81</v>
       </c>
       <c r="M679">
-        <v>39593695</v>
+        <v>39591485</v>
       </c>
       <c r="N679">
-        <v>5298694</v>
+        <v>5298145</v>
       </c>
       <c r="O679">
-        <v>2135260</v>
+        <v>2133774</v>
       </c>
       <c r="P679">
-        <v>5464</v>
+        <v>5462</v>
       </c>
       <c r="Q679">
-        <v>15173</v>
+        <v>15191</v>
       </c>
       <c r="R679">
-        <v>502034</v>
+        <v>502899</v>
       </c>
     </row>
     <row r="680">
@@ -36536,52 +36536,105 @@
         <v>46234</v>
       </c>
       <c r="B680">
-        <v>904125</v>
+        <v>882022</v>
       </c>
       <c r="C680">
         <v>1798.5</v>
       </c>
       <c r="D680">
-        <v>471790</v>
+        <v>467724</v>
       </c>
       <c r="E680">
-        <v>173460</v>
+        <v>166117</v>
       </c>
       <c r="F680">
-        <v>7806998</v>
+        <v>7594416</v>
       </c>
       <c r="G680">
-        <v>6699816</v>
+        <v>6567597</v>
       </c>
       <c r="H680">
-        <v>3156635</v>
+        <v>3107974</v>
       </c>
       <c r="I680">
-        <v>482.86</v>
+        <v>483.08</v>
       </c>
       <c r="J680">
-        <v>39.53</v>
+        <v>39.37</v>
       </c>
       <c r="K680">
-        <v>15.74</v>
+        <v>15.73</v>
       </c>
       <c r="L680">
-        <v>490.91</v>
+        <v>490.94</v>
       </c>
       <c r="M680">
-        <v>39460143</v>
+        <v>39409273</v>
       </c>
       <c r="N680">
-        <v>5260934</v>
+        <v>5256319</v>
       </c>
       <c r="O680">
-        <v>2126111</v>
+        <v>2117282</v>
       </c>
       <c r="P680">
-        <v>5471</v>
+        <v>5480</v>
       </c>
       <c r="Q680">
-        <v>15116</v>
+        <v>15129</v>
+      </c>
+      <c r="R680">
+        <v>503031</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B681">
+        <v>761770</v>
+      </c>
+      <c r="D681">
+        <v>374801</v>
+      </c>
+      <c r="E681">
+        <v>178995</v>
+      </c>
+      <c r="F681">
+        <v>8154945</v>
+      </c>
+      <c r="G681">
+        <v>6899214</v>
+      </c>
+      <c r="H681">
+        <v>3278971</v>
+      </c>
+      <c r="I681">
+        <v>486.71</v>
+      </c>
+      <c r="J681">
+        <v>39.27</v>
+      </c>
+      <c r="K681">
+        <v>15.81</v>
+      </c>
+      <c r="L681">
+        <v>493.44</v>
+      </c>
+      <c r="M681">
+        <v>39592193</v>
+      </c>
+      <c r="N681">
+        <v>5225460</v>
+      </c>
+      <c r="O681">
+        <v>2118500</v>
+      </c>
+      <c r="P681">
+        <v>5470</v>
+      </c>
+      <c r="Q681">
+        <v>15179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>